<commit_message>
Add activity_icon field to itinerary activity import
- Extend ItineraryActivityImportRow with an activityIcon column so tour
  imports can set the icon per itinerary activity
- Map the trimmed value onto the entity during import
- Regenerate the xlsx import templates to include the new column
</commit_message>
<xml_diff>
--- a/boxhilltravel-manager/src/main/resources/import-templates/tours_import_template.xlsx
+++ b/boxhilltravel-manager/src/main/resources/import-templates/tours_import_template.xlsx
@@ -666,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L251"/>
+  <dimension ref="A1:M251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -681,6 +681,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -744,6 +745,11 @@
           <t>Departure Status</t>
         </is>
       </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Activity Icon</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -781,7 +787,6 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -800,6 +805,11 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>Open</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>fa fa-camera-retro</t>
         </is>
       </c>
     </row>
@@ -864,6 +874,11 @@
           <t>Full</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>fa fa-bed</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -911,6 +926,11 @@
           <t>Ended</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>fa fa-bus</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -948,6 +968,11 @@
           <t>Cancelled</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>fa fa-coffee</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -980,6 +1005,11 @@
           <t>Rail Collection</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>fa fa-users</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1002,6 +1032,11 @@
           <t>Award Winning</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>fa fa-automobile</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1024,6 +1059,11 @@
           <t>Limited Edition</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>fa fa-ship</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1041,6 +1081,11 @@
           <t>THB</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>fa fa-cutlery</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1053,6 +1098,11 @@
           <t>IDR</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>fa fa-plane</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1065,6 +1115,11 @@
           <t>ESP</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>fa fa-train</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1077,6 +1132,11 @@
           <t>GBP</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>fa fa-car</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1089,6 +1149,11 @@
           <t>BRL</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>fa fa-suitcase</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1101,6 +1166,11 @@
           <t>MXN</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>fa fa-bicycle</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1113,6 +1183,11 @@
           <t>TRY</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>fa fa-shopping-bag</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1125,6 +1200,11 @@
           <t>ZAR</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>fa fa-taxi</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1135,6 +1215,11 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>CZK</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>fa fa-building</t>
         </is>
       </c>
     </row>
@@ -3226,8 +3311,6 @@
           <t>Visit Ho Chi Minh Mausoleum, Temple of Literature and Hoan Kiem Lake.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3263,8 +3346,6 @@
           <t>Boat trip through Trang An scenic landscape and Hoa Lu ancient capital.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3300,8 +3381,6 @@
           <t>Board an overnight cruise through the limestone karsts of Halong Bay.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3337,8 +3416,6 @@
           <t>Morning cruise activities then transfer to airport for flight to Ho Chi Minh City.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3374,8 +3451,6 @@
           <t>Explore the historic Cu Chi Tunnels and Ho Chi Minh City landmarks.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3411,8 +3486,6 @@
           <t>Free time until transfer to the airport for departure.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3457,7 +3530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3465,7 +3538,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3495,12 +3568,17 @@
           <t>description</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>activity_icon</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>subtitle</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>show_in_preview</t>
         </is>
@@ -3530,10 +3608,15 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>fa fa-camera-retro</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>classic</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3563,10 +3646,15 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>fa fa-camera-retro</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>recommand</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3596,19 +3684,27 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>fa fa-ship</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>free</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="G2:G502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
       <formula1>Lists!$I$2:$I$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>Lists!$M$2:$M$17</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>